<commit_message>
RAID Decisions sheet + template, Export PDF replaces Print, PowerPoint export on the client template
- RAID: Decisions sheet (parser, summary, UI table, KPI highlights/actions), new templates/ATS_RAID_Log_Template.xlsx, sample log gains decisions
- Replace Print with Export PDF (bundled jsPDF + html2canvas): full pack for Monthly/Weekly, current view for Programme/POAP
- PowerPoint export now sits on the client PowerPoint theme (lean embedded template: masters, layouts, logos only; no slide content), native editable charts and tables, real title placeholders and table style
- tools/build_pptx_template.py rebuilds the embedded theme from a corporate deck; docs and README updated

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/ATS_Program_SAMPLE/Self Assessment/ATS_RAID_Log.xlsx
+++ b/samples/ATS_Program_SAMPLE/Self Assessment/ATS_RAID_Log.xlsx
@@ -12,13 +12,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Guide" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Guide" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Risks'!$C$10:$T$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Issues'!$C$10:$X$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Assumptions'!$C$10:$P$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Dependencies'!$C$10:$R$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Decisions'!$C$10:$S$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8024,6 +8026,1652 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="C2:S70"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="2" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Decision Log</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>One row per decision taken - who decided, when, why and what it affects. Pending decisions show as open on the dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>SAMPLE – fictional data for demonstration only. Yellow cells are inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Summary Title</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Decision / Description</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>Decision Maker / Forum</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Date Decided</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>Rationale</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>Impact of Decision</t>
+        </is>
+      </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="L10" s="14" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="M10" s="14" t="inlineStr">
+        <is>
+          <t>Review Date</t>
+        </is>
+      </c>
+      <c r="N10" s="14" t="inlineStr">
+        <is>
+          <t>Linked Risk / Issue ID</t>
+        </is>
+      </c>
+      <c r="O10" s="14" t="inlineStr">
+        <is>
+          <t>Notes/Actions</t>
+        </is>
+      </c>
+      <c r="P10" s="14" t="inlineStr">
+        <is>
+          <t>Where Raised</t>
+        </is>
+      </c>
+      <c r="Q10" s="14" t="inlineStr">
+        <is>
+          <t>Prog RAID</t>
+        </is>
+      </c>
+      <c r="R10" s="14" t="inlineStr">
+        <is>
+          <t>Prog RAID Reference</t>
+        </is>
+      </c>
+      <c r="S10" s="14" t="inlineStr">
+        <is>
+          <t>Archived</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>DEC-001</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Adopt risk-based regression selection</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Regression scope for each release is selected by risk rather than running the full pack.</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>Test Forum</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>46273</v>
+      </c>
+      <c r="I11" s="15" t="inlineStr">
+        <is>
+          <t>Full regression no longer fits the window as the pack grows faster than capacity.</t>
+        </is>
+      </c>
+      <c r="J11" s="15" t="inlineStr">
+        <is>
+          <t>Reduced execution effort; slightly lower coverage on low-risk journeys.</t>
+        </is>
+      </c>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L11" s="15" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="M11" s="16" t="n">
+        <v>46332</v>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>R-006</t>
+        </is>
+      </c>
+      <c r="O11" s="15" t="inlineStr">
+        <is>
+          <t>Selection criteria published on the team wiki.</t>
+        </is>
+      </c>
+      <c r="P11" s="15" t="inlineStr">
+        <is>
+          <t>Test forum</t>
+        </is>
+      </c>
+      <c r="Q11" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R11" s="15" t="n"/>
+      <c r="S11" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>DEC-002</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Stub fallback for Notification Service sandbox</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>Use agreed stubs whenever the third-party sandbox is unavailable.</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>Portfolio Test Lead</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>46287</v>
+      </c>
+      <c r="I12" s="15" t="inlineStr">
+        <is>
+          <t>Sandbox availability is intermittent and blocks execution.</t>
+        </is>
+      </c>
+      <c r="J12" s="15" t="inlineStr">
+        <is>
+          <t>Faster execution; reduced confidence on live integration behaviour.</t>
+        </is>
+      </c>
+      <c r="K12" s="15" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L12" s="15" t="inlineStr">
+        <is>
+          <t>Portfolio Test Lead</t>
+        </is>
+      </c>
+      <c r="M12" s="16" t="n">
+        <v>46318</v>
+      </c>
+      <c r="N12" s="15" t="inlineStr">
+        <is>
+          <t>I-005</t>
+        </is>
+      </c>
+      <c r="O12" s="15" t="inlineStr">
+        <is>
+          <t>Revisit once sandbox is stable.</t>
+        </is>
+      </c>
+      <c r="P12" s="15" t="inlineStr">
+        <is>
+          <t>Weekly test review</t>
+        </is>
+      </c>
+      <c r="Q12" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R12" s="15" t="n"/>
+      <c r="S12" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>DEC-003</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>Move Cycle 2 start to align with vendor drop</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>Cycle 2 start moves by one week to follow the vendor build 3.2 delivery.</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>Steering Group</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>46294</v>
+      </c>
+      <c r="I13" s="15" t="inlineStr">
+        <is>
+          <t>Starting before the drop would waste execution capacity.</t>
+        </is>
+      </c>
+      <c r="J13" s="15" t="inlineStr">
+        <is>
+          <t>Cycle 2 completes one week later; still before the change freeze.</t>
+        </is>
+      </c>
+      <c r="K13" s="15" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L13" s="15" t="inlineStr">
+        <is>
+          <t>Programme Test Manager</t>
+        </is>
+      </c>
+      <c r="M13" s="16" t="n">
+        <v>46304</v>
+      </c>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>R-003</t>
+        </is>
+      </c>
+      <c r="O13" s="15" t="n"/>
+      <c r="P13" s="15" t="inlineStr">
+        <is>
+          <t>Steering group</t>
+        </is>
+      </c>
+      <c r="Q13" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R13" s="15" t="inlineStr">
+        <is>
+          <t>PR-0501</t>
+        </is>
+      </c>
+      <c r="S13" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>DEC-004</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Freeze test scope two weeks before each cycle</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>Scope changes after the freeze need a test impact assessment and change board approval.</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>Change Board</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="n">
+        <v>46280</v>
+      </c>
+      <c r="I14" s="15" t="inlineStr">
+        <is>
+          <t>Late changes caused rework of scripts and data.</t>
+        </is>
+      </c>
+      <c r="J14" s="15" t="inlineStr">
+        <is>
+          <t>Greater stability; slower acceptance of late scope.</t>
+        </is>
+      </c>
+      <c r="K14" s="15" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L14" s="15" t="inlineStr">
+        <is>
+          <t>Portfolio Test Lead</t>
+        </is>
+      </c>
+      <c r="M14" s="16" t="n">
+        <v>46325</v>
+      </c>
+      <c r="N14" s="15" t="inlineStr">
+        <is>
+          <t>R-005</t>
+        </is>
+      </c>
+      <c r="O14" s="15" t="n"/>
+      <c r="P14" s="15" t="inlineStr">
+        <is>
+          <t>Change board</t>
+        </is>
+      </c>
+      <c r="Q14" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R14" s="15" t="n"/>
+      <c r="S14" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>DEC-005</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>Add two analysts for Cycle 2</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>Request two additional test analysts to cover the execution shortfall.</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>Resourcing</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>Programme Test Manager</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="n"/>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>Capacity model shows a shortfall in Cycle 2.</t>
+        </is>
+      </c>
+      <c r="J15" s="15" t="inlineStr">
+        <is>
+          <t>Closes the capacity gap; additional cost.</t>
+        </is>
+      </c>
+      <c r="K15" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L15" s="15" t="inlineStr">
+        <is>
+          <t>Programme Test Manager</t>
+        </is>
+      </c>
+      <c r="M15" s="16" t="n">
+        <v>46311</v>
+      </c>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>D-006</t>
+        </is>
+      </c>
+      <c r="O15" s="15" t="inlineStr">
+        <is>
+          <t>Awaiting commercial approval.</t>
+        </is>
+      </c>
+      <c r="P15" s="15" t="inlineStr">
+        <is>
+          <t>Resourcing review</t>
+        </is>
+      </c>
+      <c r="Q15" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R15" s="15" t="n"/>
+      <c r="S15" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>DEC-006</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Retire manual smoke pack in favour of automated pack</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>Manual smoke checks are replaced by the automated smoke suite.</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>Test Forum</t>
+        </is>
+      </c>
+      <c r="H16" s="16" t="n">
+        <v>46252</v>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>Automated pack now covers all smoke journeys.</t>
+        </is>
+      </c>
+      <c r="J16" s="15" t="inlineStr">
+        <is>
+          <t>Saves around two days per release.</t>
+        </is>
+      </c>
+      <c r="K16" s="15" t="inlineStr">
+        <is>
+          <t>Superseded</t>
+        </is>
+      </c>
+      <c r="L16" s="15" t="inlineStr">
+        <is>
+          <t>Test Manager</t>
+        </is>
+      </c>
+      <c r="M16" s="16" t="n"/>
+      <c r="N16" s="15" t="n"/>
+      <c r="O16" s="15" t="inlineStr">
+        <is>
+          <t>Superseded by risk-based selection decision D-001.</t>
+        </is>
+      </c>
+      <c r="P16" s="15" t="inlineStr">
+        <is>
+          <t>Test forum</t>
+        </is>
+      </c>
+      <c r="Q16" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R16" s="15" t="n"/>
+      <c r="S16" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="16" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="15" t="n"/>
+      <c r="K17" s="15" t="n"/>
+      <c r="L17" s="15" t="n"/>
+      <c r="M17" s="16" t="n"/>
+      <c r="N17" s="15" t="n"/>
+      <c r="O17" s="15" t="n"/>
+      <c r="P17" s="15" t="n"/>
+      <c r="Q17" s="15" t="n"/>
+      <c r="R17" s="15" t="n"/>
+      <c r="S17" s="15" t="n"/>
+    </row>
+    <row r="18">
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="16" t="n"/>
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="n"/>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="16" t="n"/>
+      <c r="N18" s="15" t="n"/>
+      <c r="O18" s="15" t="n"/>
+      <c r="P18" s="15" t="n"/>
+      <c r="Q18" s="15" t="n"/>
+      <c r="R18" s="15" t="n"/>
+      <c r="S18" s="15" t="n"/>
+    </row>
+    <row r="19">
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="16" t="n"/>
+      <c r="I19" s="15" t="n"/>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="15" t="n"/>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="16" t="n"/>
+      <c r="N19" s="15" t="n"/>
+      <c r="O19" s="15" t="n"/>
+      <c r="P19" s="15" t="n"/>
+      <c r="Q19" s="15" t="n"/>
+      <c r="R19" s="15" t="n"/>
+      <c r="S19" s="15" t="n"/>
+    </row>
+    <row r="20">
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="15" t="n"/>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="16" t="n"/>
+      <c r="I20" s="15" t="n"/>
+      <c r="J20" s="15" t="n"/>
+      <c r="K20" s="15" t="n"/>
+      <c r="L20" s="15" t="n"/>
+      <c r="M20" s="16" t="n"/>
+      <c r="N20" s="15" t="n"/>
+      <c r="O20" s="15" t="n"/>
+      <c r="P20" s="15" t="n"/>
+      <c r="Q20" s="15" t="n"/>
+      <c r="R20" s="15" t="n"/>
+      <c r="S20" s="15" t="n"/>
+    </row>
+    <row r="21">
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15" t="n"/>
+      <c r="G21" s="15" t="n"/>
+      <c r="H21" s="16" t="n"/>
+      <c r="I21" s="15" t="n"/>
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
+      <c r="L21" s="15" t="n"/>
+      <c r="M21" s="16" t="n"/>
+      <c r="N21" s="15" t="n"/>
+      <c r="O21" s="15" t="n"/>
+      <c r="P21" s="15" t="n"/>
+      <c r="Q21" s="15" t="n"/>
+      <c r="R21" s="15" t="n"/>
+      <c r="S21" s="15" t="n"/>
+    </row>
+    <row r="22">
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="15" t="n"/>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="16" t="n"/>
+      <c r="I22" s="15" t="n"/>
+      <c r="J22" s="15" t="n"/>
+      <c r="K22" s="15" t="n"/>
+      <c r="L22" s="15" t="n"/>
+      <c r="M22" s="16" t="n"/>
+      <c r="N22" s="15" t="n"/>
+      <c r="O22" s="15" t="n"/>
+      <c r="P22" s="15" t="n"/>
+      <c r="Q22" s="15" t="n"/>
+      <c r="R22" s="15" t="n"/>
+      <c r="S22" s="15" t="n"/>
+    </row>
+    <row r="23">
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="16" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
+      <c r="M23" s="16" t="n"/>
+      <c r="N23" s="15" t="n"/>
+      <c r="O23" s="15" t="n"/>
+      <c r="P23" s="15" t="n"/>
+      <c r="Q23" s="15" t="n"/>
+      <c r="R23" s="15" t="n"/>
+      <c r="S23" s="15" t="n"/>
+    </row>
+    <row r="24">
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="16" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="J24" s="15" t="n"/>
+      <c r="K24" s="15" t="n"/>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="16" t="n"/>
+      <c r="N24" s="15" t="n"/>
+      <c r="O24" s="15" t="n"/>
+      <c r="P24" s="15" t="n"/>
+      <c r="Q24" s="15" t="n"/>
+      <c r="R24" s="15" t="n"/>
+      <c r="S24" s="15" t="n"/>
+    </row>
+    <row r="25">
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="15" t="n"/>
+      <c r="E25" s="15" t="n"/>
+      <c r="F25" s="15" t="n"/>
+      <c r="G25" s="15" t="n"/>
+      <c r="H25" s="16" t="n"/>
+      <c r="I25" s="15" t="n"/>
+      <c r="J25" s="15" t="n"/>
+      <c r="K25" s="15" t="n"/>
+      <c r="L25" s="15" t="n"/>
+      <c r="M25" s="16" t="n"/>
+      <c r="N25" s="15" t="n"/>
+      <c r="O25" s="15" t="n"/>
+      <c r="P25" s="15" t="n"/>
+      <c r="Q25" s="15" t="n"/>
+      <c r="R25" s="15" t="n"/>
+      <c r="S25" s="15" t="n"/>
+    </row>
+    <row r="26">
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="15" t="n"/>
+      <c r="G26" s="15" t="n"/>
+      <c r="H26" s="16" t="n"/>
+      <c r="I26" s="15" t="n"/>
+      <c r="J26" s="15" t="n"/>
+      <c r="K26" s="15" t="n"/>
+      <c r="L26" s="15" t="n"/>
+      <c r="M26" s="16" t="n"/>
+      <c r="N26" s="15" t="n"/>
+      <c r="O26" s="15" t="n"/>
+      <c r="P26" s="15" t="n"/>
+      <c r="Q26" s="15" t="n"/>
+      <c r="R26" s="15" t="n"/>
+      <c r="S26" s="15" t="n"/>
+    </row>
+    <row r="27">
+      <c r="C27" s="15" t="n"/>
+      <c r="D27" s="15" t="n"/>
+      <c r="E27" s="15" t="n"/>
+      <c r="F27" s="15" t="n"/>
+      <c r="G27" s="15" t="n"/>
+      <c r="H27" s="16" t="n"/>
+      <c r="I27" s="15" t="n"/>
+      <c r="J27" s="15" t="n"/>
+      <c r="K27" s="15" t="n"/>
+      <c r="L27" s="15" t="n"/>
+      <c r="M27" s="16" t="n"/>
+      <c r="N27" s="15" t="n"/>
+      <c r="O27" s="15" t="n"/>
+      <c r="P27" s="15" t="n"/>
+      <c r="Q27" s="15" t="n"/>
+      <c r="R27" s="15" t="n"/>
+      <c r="S27" s="15" t="n"/>
+    </row>
+    <row r="28">
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="15" t="n"/>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="16" t="n"/>
+      <c r="I28" s="15" t="n"/>
+      <c r="J28" s="15" t="n"/>
+      <c r="K28" s="15" t="n"/>
+      <c r="L28" s="15" t="n"/>
+      <c r="M28" s="16" t="n"/>
+      <c r="N28" s="15" t="n"/>
+      <c r="O28" s="15" t="n"/>
+      <c r="P28" s="15" t="n"/>
+      <c r="Q28" s="15" t="n"/>
+      <c r="R28" s="15" t="n"/>
+      <c r="S28" s="15" t="n"/>
+    </row>
+    <row r="29">
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="15" t="n"/>
+      <c r="G29" s="15" t="n"/>
+      <c r="H29" s="16" t="n"/>
+      <c r="I29" s="15" t="n"/>
+      <c r="J29" s="15" t="n"/>
+      <c r="K29" s="15" t="n"/>
+      <c r="L29" s="15" t="n"/>
+      <c r="M29" s="16" t="n"/>
+      <c r="N29" s="15" t="n"/>
+      <c r="O29" s="15" t="n"/>
+      <c r="P29" s="15" t="n"/>
+      <c r="Q29" s="15" t="n"/>
+      <c r="R29" s="15" t="n"/>
+      <c r="S29" s="15" t="n"/>
+    </row>
+    <row r="30">
+      <c r="C30" s="15" t="n"/>
+      <c r="D30" s="15" t="n"/>
+      <c r="E30" s="15" t="n"/>
+      <c r="F30" s="15" t="n"/>
+      <c r="G30" s="15" t="n"/>
+      <c r="H30" s="16" t="n"/>
+      <c r="I30" s="15" t="n"/>
+      <c r="J30" s="15" t="n"/>
+      <c r="K30" s="15" t="n"/>
+      <c r="L30" s="15" t="n"/>
+      <c r="M30" s="16" t="n"/>
+      <c r="N30" s="15" t="n"/>
+      <c r="O30" s="15" t="n"/>
+      <c r="P30" s="15" t="n"/>
+      <c r="Q30" s="15" t="n"/>
+      <c r="R30" s="15" t="n"/>
+      <c r="S30" s="15" t="n"/>
+    </row>
+    <row r="31">
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="15" t="n"/>
+      <c r="F31" s="15" t="n"/>
+      <c r="G31" s="15" t="n"/>
+      <c r="H31" s="16" t="n"/>
+      <c r="I31" s="15" t="n"/>
+      <c r="J31" s="15" t="n"/>
+      <c r="K31" s="15" t="n"/>
+      <c r="L31" s="15" t="n"/>
+      <c r="M31" s="16" t="n"/>
+      <c r="N31" s="15" t="n"/>
+      <c r="O31" s="15" t="n"/>
+      <c r="P31" s="15" t="n"/>
+      <c r="Q31" s="15" t="n"/>
+      <c r="R31" s="15" t="n"/>
+      <c r="S31" s="15" t="n"/>
+    </row>
+    <row r="32">
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="16" t="n"/>
+      <c r="I32" s="15" t="n"/>
+      <c r="J32" s="15" t="n"/>
+      <c r="K32" s="15" t="n"/>
+      <c r="L32" s="15" t="n"/>
+      <c r="M32" s="16" t="n"/>
+      <c r="N32" s="15" t="n"/>
+      <c r="O32" s="15" t="n"/>
+      <c r="P32" s="15" t="n"/>
+      <c r="Q32" s="15" t="n"/>
+      <c r="R32" s="15" t="n"/>
+      <c r="S32" s="15" t="n"/>
+    </row>
+    <row r="33">
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="15" t="n"/>
+      <c r="E33" s="15" t="n"/>
+      <c r="F33" s="15" t="n"/>
+      <c r="G33" s="15" t="n"/>
+      <c r="H33" s="16" t="n"/>
+      <c r="I33" s="15" t="n"/>
+      <c r="J33" s="15" t="n"/>
+      <c r="K33" s="15" t="n"/>
+      <c r="L33" s="15" t="n"/>
+      <c r="M33" s="16" t="n"/>
+      <c r="N33" s="15" t="n"/>
+      <c r="O33" s="15" t="n"/>
+      <c r="P33" s="15" t="n"/>
+      <c r="Q33" s="15" t="n"/>
+      <c r="R33" s="15" t="n"/>
+      <c r="S33" s="15" t="n"/>
+    </row>
+    <row r="34">
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="15" t="n"/>
+      <c r="G34" s="15" t="n"/>
+      <c r="H34" s="16" t="n"/>
+      <c r="I34" s="15" t="n"/>
+      <c r="J34" s="15" t="n"/>
+      <c r="K34" s="15" t="n"/>
+      <c r="L34" s="15" t="n"/>
+      <c r="M34" s="16" t="n"/>
+      <c r="N34" s="15" t="n"/>
+      <c r="O34" s="15" t="n"/>
+      <c r="P34" s="15" t="n"/>
+      <c r="Q34" s="15" t="n"/>
+      <c r="R34" s="15" t="n"/>
+      <c r="S34" s="15" t="n"/>
+    </row>
+    <row r="35">
+      <c r="C35" s="15" t="n"/>
+      <c r="D35" s="15" t="n"/>
+      <c r="E35" s="15" t="n"/>
+      <c r="F35" s="15" t="n"/>
+      <c r="G35" s="15" t="n"/>
+      <c r="H35" s="16" t="n"/>
+      <c r="I35" s="15" t="n"/>
+      <c r="J35" s="15" t="n"/>
+      <c r="K35" s="15" t="n"/>
+      <c r="L35" s="15" t="n"/>
+      <c r="M35" s="16" t="n"/>
+      <c r="N35" s="15" t="n"/>
+      <c r="O35" s="15" t="n"/>
+      <c r="P35" s="15" t="n"/>
+      <c r="Q35" s="15" t="n"/>
+      <c r="R35" s="15" t="n"/>
+      <c r="S35" s="15" t="n"/>
+    </row>
+    <row r="36">
+      <c r="C36" s="15" t="n"/>
+      <c r="D36" s="15" t="n"/>
+      <c r="E36" s="15" t="n"/>
+      <c r="F36" s="15" t="n"/>
+      <c r="G36" s="15" t="n"/>
+      <c r="H36" s="16" t="n"/>
+      <c r="I36" s="15" t="n"/>
+      <c r="J36" s="15" t="n"/>
+      <c r="K36" s="15" t="n"/>
+      <c r="L36" s="15" t="n"/>
+      <c r="M36" s="16" t="n"/>
+      <c r="N36" s="15" t="n"/>
+      <c r="O36" s="15" t="n"/>
+      <c r="P36" s="15" t="n"/>
+      <c r="Q36" s="15" t="n"/>
+      <c r="R36" s="15" t="n"/>
+      <c r="S36" s="15" t="n"/>
+    </row>
+    <row r="37">
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="15" t="n"/>
+      <c r="F37" s="15" t="n"/>
+      <c r="G37" s="15" t="n"/>
+      <c r="H37" s="16" t="n"/>
+      <c r="I37" s="15" t="n"/>
+      <c r="J37" s="15" t="n"/>
+      <c r="K37" s="15" t="n"/>
+      <c r="L37" s="15" t="n"/>
+      <c r="M37" s="16" t="n"/>
+      <c r="N37" s="15" t="n"/>
+      <c r="O37" s="15" t="n"/>
+      <c r="P37" s="15" t="n"/>
+      <c r="Q37" s="15" t="n"/>
+      <c r="R37" s="15" t="n"/>
+      <c r="S37" s="15" t="n"/>
+    </row>
+    <row r="38">
+      <c r="C38" s="15" t="n"/>
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="15" t="n"/>
+      <c r="F38" s="15" t="n"/>
+      <c r="G38" s="15" t="n"/>
+      <c r="H38" s="16" t="n"/>
+      <c r="I38" s="15" t="n"/>
+      <c r="J38" s="15" t="n"/>
+      <c r="K38" s="15" t="n"/>
+      <c r="L38" s="15" t="n"/>
+      <c r="M38" s="16" t="n"/>
+      <c r="N38" s="15" t="n"/>
+      <c r="O38" s="15" t="n"/>
+      <c r="P38" s="15" t="n"/>
+      <c r="Q38" s="15" t="n"/>
+      <c r="R38" s="15" t="n"/>
+      <c r="S38" s="15" t="n"/>
+    </row>
+    <row r="39">
+      <c r="C39" s="15" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="15" t="n"/>
+      <c r="F39" s="15" t="n"/>
+      <c r="G39" s="15" t="n"/>
+      <c r="H39" s="16" t="n"/>
+      <c r="I39" s="15" t="n"/>
+      <c r="J39" s="15" t="n"/>
+      <c r="K39" s="15" t="n"/>
+      <c r="L39" s="15" t="n"/>
+      <c r="M39" s="16" t="n"/>
+      <c r="N39" s="15" t="n"/>
+      <c r="O39" s="15" t="n"/>
+      <c r="P39" s="15" t="n"/>
+      <c r="Q39" s="15" t="n"/>
+      <c r="R39" s="15" t="n"/>
+      <c r="S39" s="15" t="n"/>
+    </row>
+    <row r="40">
+      <c r="C40" s="15" t="n"/>
+      <c r="D40" s="15" t="n"/>
+      <c r="E40" s="15" t="n"/>
+      <c r="F40" s="15" t="n"/>
+      <c r="G40" s="15" t="n"/>
+      <c r="H40" s="16" t="n"/>
+      <c r="I40" s="15" t="n"/>
+      <c r="J40" s="15" t="n"/>
+      <c r="K40" s="15" t="n"/>
+      <c r="L40" s="15" t="n"/>
+      <c r="M40" s="16" t="n"/>
+      <c r="N40" s="15" t="n"/>
+      <c r="O40" s="15" t="n"/>
+      <c r="P40" s="15" t="n"/>
+      <c r="Q40" s="15" t="n"/>
+      <c r="R40" s="15" t="n"/>
+      <c r="S40" s="15" t="n"/>
+    </row>
+    <row r="41">
+      <c r="C41" s="15" t="n"/>
+      <c r="D41" s="15" t="n"/>
+      <c r="E41" s="15" t="n"/>
+      <c r="F41" s="15" t="n"/>
+      <c r="G41" s="15" t="n"/>
+      <c r="H41" s="16" t="n"/>
+      <c r="I41" s="15" t="n"/>
+      <c r="J41" s="15" t="n"/>
+      <c r="K41" s="15" t="n"/>
+      <c r="L41" s="15" t="n"/>
+      <c r="M41" s="16" t="n"/>
+      <c r="N41" s="15" t="n"/>
+      <c r="O41" s="15" t="n"/>
+      <c r="P41" s="15" t="n"/>
+      <c r="Q41" s="15" t="n"/>
+      <c r="R41" s="15" t="n"/>
+      <c r="S41" s="15" t="n"/>
+    </row>
+    <row r="42">
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="15" t="n"/>
+      <c r="F42" s="15" t="n"/>
+      <c r="G42" s="15" t="n"/>
+      <c r="H42" s="16" t="n"/>
+      <c r="I42" s="15" t="n"/>
+      <c r="J42" s="15" t="n"/>
+      <c r="K42" s="15" t="n"/>
+      <c r="L42" s="15" t="n"/>
+      <c r="M42" s="16" t="n"/>
+      <c r="N42" s="15" t="n"/>
+      <c r="O42" s="15" t="n"/>
+      <c r="P42" s="15" t="n"/>
+      <c r="Q42" s="15" t="n"/>
+      <c r="R42" s="15" t="n"/>
+      <c r="S42" s="15" t="n"/>
+    </row>
+    <row r="43">
+      <c r="C43" s="15" t="n"/>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="15" t="n"/>
+      <c r="F43" s="15" t="n"/>
+      <c r="G43" s="15" t="n"/>
+      <c r="H43" s="16" t="n"/>
+      <c r="I43" s="15" t="n"/>
+      <c r="J43" s="15" t="n"/>
+      <c r="K43" s="15" t="n"/>
+      <c r="L43" s="15" t="n"/>
+      <c r="M43" s="16" t="n"/>
+      <c r="N43" s="15" t="n"/>
+      <c r="O43" s="15" t="n"/>
+      <c r="P43" s="15" t="n"/>
+      <c r="Q43" s="15" t="n"/>
+      <c r="R43" s="15" t="n"/>
+      <c r="S43" s="15" t="n"/>
+    </row>
+    <row r="44">
+      <c r="C44" s="15" t="n"/>
+      <c r="D44" s="15" t="n"/>
+      <c r="E44" s="15" t="n"/>
+      <c r="F44" s="15" t="n"/>
+      <c r="G44" s="15" t="n"/>
+      <c r="H44" s="16" t="n"/>
+      <c r="I44" s="15" t="n"/>
+      <c r="J44" s="15" t="n"/>
+      <c r="K44" s="15" t="n"/>
+      <c r="L44" s="15" t="n"/>
+      <c r="M44" s="16" t="n"/>
+      <c r="N44" s="15" t="n"/>
+      <c r="O44" s="15" t="n"/>
+      <c r="P44" s="15" t="n"/>
+      <c r="Q44" s="15" t="n"/>
+      <c r="R44" s="15" t="n"/>
+      <c r="S44" s="15" t="n"/>
+    </row>
+    <row r="45">
+      <c r="C45" s="15" t="n"/>
+      <c r="D45" s="15" t="n"/>
+      <c r="E45" s="15" t="n"/>
+      <c r="F45" s="15" t="n"/>
+      <c r="G45" s="15" t="n"/>
+      <c r="H45" s="16" t="n"/>
+      <c r="I45" s="15" t="n"/>
+      <c r="J45" s="15" t="n"/>
+      <c r="K45" s="15" t="n"/>
+      <c r="L45" s="15" t="n"/>
+      <c r="M45" s="16" t="n"/>
+      <c r="N45" s="15" t="n"/>
+      <c r="O45" s="15" t="n"/>
+      <c r="P45" s="15" t="n"/>
+      <c r="Q45" s="15" t="n"/>
+      <c r="R45" s="15" t="n"/>
+      <c r="S45" s="15" t="n"/>
+    </row>
+    <row r="46">
+      <c r="C46" s="15" t="n"/>
+      <c r="D46" s="15" t="n"/>
+      <c r="E46" s="15" t="n"/>
+      <c r="F46" s="15" t="n"/>
+      <c r="G46" s="15" t="n"/>
+      <c r="H46" s="16" t="n"/>
+      <c r="I46" s="15" t="n"/>
+      <c r="J46" s="15" t="n"/>
+      <c r="K46" s="15" t="n"/>
+      <c r="L46" s="15" t="n"/>
+      <c r="M46" s="16" t="n"/>
+      <c r="N46" s="15" t="n"/>
+      <c r="O46" s="15" t="n"/>
+      <c r="P46" s="15" t="n"/>
+      <c r="Q46" s="15" t="n"/>
+      <c r="R46" s="15" t="n"/>
+      <c r="S46" s="15" t="n"/>
+    </row>
+    <row r="47">
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="15" t="n"/>
+      <c r="F47" s="15" t="n"/>
+      <c r="G47" s="15" t="n"/>
+      <c r="H47" s="16" t="n"/>
+      <c r="I47" s="15" t="n"/>
+      <c r="J47" s="15" t="n"/>
+      <c r="K47" s="15" t="n"/>
+      <c r="L47" s="15" t="n"/>
+      <c r="M47" s="16" t="n"/>
+      <c r="N47" s="15" t="n"/>
+      <c r="O47" s="15" t="n"/>
+      <c r="P47" s="15" t="n"/>
+      <c r="Q47" s="15" t="n"/>
+      <c r="R47" s="15" t="n"/>
+      <c r="S47" s="15" t="n"/>
+    </row>
+    <row r="48">
+      <c r="C48" s="15" t="n"/>
+      <c r="D48" s="15" t="n"/>
+      <c r="E48" s="15" t="n"/>
+      <c r="F48" s="15" t="n"/>
+      <c r="G48" s="15" t="n"/>
+      <c r="H48" s="16" t="n"/>
+      <c r="I48" s="15" t="n"/>
+      <c r="J48" s="15" t="n"/>
+      <c r="K48" s="15" t="n"/>
+      <c r="L48" s="15" t="n"/>
+      <c r="M48" s="16" t="n"/>
+      <c r="N48" s="15" t="n"/>
+      <c r="O48" s="15" t="n"/>
+      <c r="P48" s="15" t="n"/>
+      <c r="Q48" s="15" t="n"/>
+      <c r="R48" s="15" t="n"/>
+      <c r="S48" s="15" t="n"/>
+    </row>
+    <row r="49">
+      <c r="C49" s="15" t="n"/>
+      <c r="D49" s="15" t="n"/>
+      <c r="E49" s="15" t="n"/>
+      <c r="F49" s="15" t="n"/>
+      <c r="G49" s="15" t="n"/>
+      <c r="H49" s="16" t="n"/>
+      <c r="I49" s="15" t="n"/>
+      <c r="J49" s="15" t="n"/>
+      <c r="K49" s="15" t="n"/>
+      <c r="L49" s="15" t="n"/>
+      <c r="M49" s="16" t="n"/>
+      <c r="N49" s="15" t="n"/>
+      <c r="O49" s="15" t="n"/>
+      <c r="P49" s="15" t="n"/>
+      <c r="Q49" s="15" t="n"/>
+      <c r="R49" s="15" t="n"/>
+      <c r="S49" s="15" t="n"/>
+    </row>
+    <row r="50">
+      <c r="C50" s="15" t="n"/>
+      <c r="D50" s="15" t="n"/>
+      <c r="E50" s="15" t="n"/>
+      <c r="F50" s="15" t="n"/>
+      <c r="G50" s="15" t="n"/>
+      <c r="H50" s="16" t="n"/>
+      <c r="I50" s="15" t="n"/>
+      <c r="J50" s="15" t="n"/>
+      <c r="K50" s="15" t="n"/>
+      <c r="L50" s="15" t="n"/>
+      <c r="M50" s="16" t="n"/>
+      <c r="N50" s="15" t="n"/>
+      <c r="O50" s="15" t="n"/>
+      <c r="P50" s="15" t="n"/>
+      <c r="Q50" s="15" t="n"/>
+      <c r="R50" s="15" t="n"/>
+      <c r="S50" s="15" t="n"/>
+    </row>
+    <row r="51">
+      <c r="C51" s="15" t="n"/>
+      <c r="D51" s="15" t="n"/>
+      <c r="E51" s="15" t="n"/>
+      <c r="F51" s="15" t="n"/>
+      <c r="G51" s="15" t="n"/>
+      <c r="H51" s="16" t="n"/>
+      <c r="I51" s="15" t="n"/>
+      <c r="J51" s="15" t="n"/>
+      <c r="K51" s="15" t="n"/>
+      <c r="L51" s="15" t="n"/>
+      <c r="M51" s="16" t="n"/>
+      <c r="N51" s="15" t="n"/>
+      <c r="O51" s="15" t="n"/>
+      <c r="P51" s="15" t="n"/>
+      <c r="Q51" s="15" t="n"/>
+      <c r="R51" s="15" t="n"/>
+      <c r="S51" s="15" t="n"/>
+    </row>
+    <row r="52">
+      <c r="C52" s="15" t="n"/>
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="15" t="n"/>
+      <c r="F52" s="15" t="n"/>
+      <c r="G52" s="15" t="n"/>
+      <c r="H52" s="16" t="n"/>
+      <c r="I52" s="15" t="n"/>
+      <c r="J52" s="15" t="n"/>
+      <c r="K52" s="15" t="n"/>
+      <c r="L52" s="15" t="n"/>
+      <c r="M52" s="16" t="n"/>
+      <c r="N52" s="15" t="n"/>
+      <c r="O52" s="15" t="n"/>
+      <c r="P52" s="15" t="n"/>
+      <c r="Q52" s="15" t="n"/>
+      <c r="R52" s="15" t="n"/>
+      <c r="S52" s="15" t="n"/>
+    </row>
+    <row r="53">
+      <c r="C53" s="15" t="n"/>
+      <c r="D53" s="15" t="n"/>
+      <c r="E53" s="15" t="n"/>
+      <c r="F53" s="15" t="n"/>
+      <c r="G53" s="15" t="n"/>
+      <c r="H53" s="16" t="n"/>
+      <c r="I53" s="15" t="n"/>
+      <c r="J53" s="15" t="n"/>
+      <c r="K53" s="15" t="n"/>
+      <c r="L53" s="15" t="n"/>
+      <c r="M53" s="16" t="n"/>
+      <c r="N53" s="15" t="n"/>
+      <c r="O53" s="15" t="n"/>
+      <c r="P53" s="15" t="n"/>
+      <c r="Q53" s="15" t="n"/>
+      <c r="R53" s="15" t="n"/>
+      <c r="S53" s="15" t="n"/>
+    </row>
+    <row r="54">
+      <c r="C54" s="15" t="n"/>
+      <c r="D54" s="15" t="n"/>
+      <c r="E54" s="15" t="n"/>
+      <c r="F54" s="15" t="n"/>
+      <c r="G54" s="15" t="n"/>
+      <c r="H54" s="16" t="n"/>
+      <c r="I54" s="15" t="n"/>
+      <c r="J54" s="15" t="n"/>
+      <c r="K54" s="15" t="n"/>
+      <c r="L54" s="15" t="n"/>
+      <c r="M54" s="16" t="n"/>
+      <c r="N54" s="15" t="n"/>
+      <c r="O54" s="15" t="n"/>
+      <c r="P54" s="15" t="n"/>
+      <c r="Q54" s="15" t="n"/>
+      <c r="R54" s="15" t="n"/>
+      <c r="S54" s="15" t="n"/>
+    </row>
+    <row r="55">
+      <c r="C55" s="15" t="n"/>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="15" t="n"/>
+      <c r="F55" s="15" t="n"/>
+      <c r="G55" s="15" t="n"/>
+      <c r="H55" s="16" t="n"/>
+      <c r="I55" s="15" t="n"/>
+      <c r="J55" s="15" t="n"/>
+      <c r="K55" s="15" t="n"/>
+      <c r="L55" s="15" t="n"/>
+      <c r="M55" s="16" t="n"/>
+      <c r="N55" s="15" t="n"/>
+      <c r="O55" s="15" t="n"/>
+      <c r="P55" s="15" t="n"/>
+      <c r="Q55" s="15" t="n"/>
+      <c r="R55" s="15" t="n"/>
+      <c r="S55" s="15" t="n"/>
+    </row>
+    <row r="56">
+      <c r="C56" s="15" t="n"/>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="15" t="n"/>
+      <c r="F56" s="15" t="n"/>
+      <c r="G56" s="15" t="n"/>
+      <c r="H56" s="16" t="n"/>
+      <c r="I56" s="15" t="n"/>
+      <c r="J56" s="15" t="n"/>
+      <c r="K56" s="15" t="n"/>
+      <c r="L56" s="15" t="n"/>
+      <c r="M56" s="16" t="n"/>
+      <c r="N56" s="15" t="n"/>
+      <c r="O56" s="15" t="n"/>
+      <c r="P56" s="15" t="n"/>
+      <c r="Q56" s="15" t="n"/>
+      <c r="R56" s="15" t="n"/>
+      <c r="S56" s="15" t="n"/>
+    </row>
+    <row r="57">
+      <c r="C57" s="15" t="n"/>
+      <c r="D57" s="15" t="n"/>
+      <c r="E57" s="15" t="n"/>
+      <c r="F57" s="15" t="n"/>
+      <c r="G57" s="15" t="n"/>
+      <c r="H57" s="16" t="n"/>
+      <c r="I57" s="15" t="n"/>
+      <c r="J57" s="15" t="n"/>
+      <c r="K57" s="15" t="n"/>
+      <c r="L57" s="15" t="n"/>
+      <c r="M57" s="16" t="n"/>
+      <c r="N57" s="15" t="n"/>
+      <c r="O57" s="15" t="n"/>
+      <c r="P57" s="15" t="n"/>
+      <c r="Q57" s="15" t="n"/>
+      <c r="R57" s="15" t="n"/>
+      <c r="S57" s="15" t="n"/>
+    </row>
+    <row r="58">
+      <c r="C58" s="15" t="n"/>
+      <c r="D58" s="15" t="n"/>
+      <c r="E58" s="15" t="n"/>
+      <c r="F58" s="15" t="n"/>
+      <c r="G58" s="15" t="n"/>
+      <c r="H58" s="16" t="n"/>
+      <c r="I58" s="15" t="n"/>
+      <c r="J58" s="15" t="n"/>
+      <c r="K58" s="15" t="n"/>
+      <c r="L58" s="15" t="n"/>
+      <c r="M58" s="16" t="n"/>
+      <c r="N58" s="15" t="n"/>
+      <c r="O58" s="15" t="n"/>
+      <c r="P58" s="15" t="n"/>
+      <c r="Q58" s="15" t="n"/>
+      <c r="R58" s="15" t="n"/>
+      <c r="S58" s="15" t="n"/>
+    </row>
+    <row r="59">
+      <c r="C59" s="15" t="n"/>
+      <c r="D59" s="15" t="n"/>
+      <c r="E59" s="15" t="n"/>
+      <c r="F59" s="15" t="n"/>
+      <c r="G59" s="15" t="n"/>
+      <c r="H59" s="16" t="n"/>
+      <c r="I59" s="15" t="n"/>
+      <c r="J59" s="15" t="n"/>
+      <c r="K59" s="15" t="n"/>
+      <c r="L59" s="15" t="n"/>
+      <c r="M59" s="16" t="n"/>
+      <c r="N59" s="15" t="n"/>
+      <c r="O59" s="15" t="n"/>
+      <c r="P59" s="15" t="n"/>
+      <c r="Q59" s="15" t="n"/>
+      <c r="R59" s="15" t="n"/>
+      <c r="S59" s="15" t="n"/>
+    </row>
+    <row r="60">
+      <c r="C60" s="15" t="n"/>
+      <c r="D60" s="15" t="n"/>
+      <c r="E60" s="15" t="n"/>
+      <c r="F60" s="15" t="n"/>
+      <c r="G60" s="15" t="n"/>
+      <c r="H60" s="16" t="n"/>
+      <c r="I60" s="15" t="n"/>
+      <c r="J60" s="15" t="n"/>
+      <c r="K60" s="15" t="n"/>
+      <c r="L60" s="15" t="n"/>
+      <c r="M60" s="16" t="n"/>
+      <c r="N60" s="15" t="n"/>
+      <c r="O60" s="15" t="n"/>
+      <c r="P60" s="15" t="n"/>
+      <c r="Q60" s="15" t="n"/>
+      <c r="R60" s="15" t="n"/>
+      <c r="S60" s="15" t="n"/>
+    </row>
+    <row r="61">
+      <c r="C61" s="15" t="n"/>
+      <c r="D61" s="15" t="n"/>
+      <c r="E61" s="15" t="n"/>
+      <c r="F61" s="15" t="n"/>
+      <c r="G61" s="15" t="n"/>
+      <c r="H61" s="16" t="n"/>
+      <c r="I61" s="15" t="n"/>
+      <c r="J61" s="15" t="n"/>
+      <c r="K61" s="15" t="n"/>
+      <c r="L61" s="15" t="n"/>
+      <c r="M61" s="16" t="n"/>
+      <c r="N61" s="15" t="n"/>
+      <c r="O61" s="15" t="n"/>
+      <c r="P61" s="15" t="n"/>
+      <c r="Q61" s="15" t="n"/>
+      <c r="R61" s="15" t="n"/>
+      <c r="S61" s="15" t="n"/>
+    </row>
+    <row r="62">
+      <c r="C62" s="15" t="n"/>
+      <c r="D62" s="15" t="n"/>
+      <c r="E62" s="15" t="n"/>
+      <c r="F62" s="15" t="n"/>
+      <c r="G62" s="15" t="n"/>
+      <c r="H62" s="16" t="n"/>
+      <c r="I62" s="15" t="n"/>
+      <c r="J62" s="15" t="n"/>
+      <c r="K62" s="15" t="n"/>
+      <c r="L62" s="15" t="n"/>
+      <c r="M62" s="16" t="n"/>
+      <c r="N62" s="15" t="n"/>
+      <c r="O62" s="15" t="n"/>
+      <c r="P62" s="15" t="n"/>
+      <c r="Q62" s="15" t="n"/>
+      <c r="R62" s="15" t="n"/>
+      <c r="S62" s="15" t="n"/>
+    </row>
+    <row r="63">
+      <c r="C63" s="15" t="n"/>
+      <c r="D63" s="15" t="n"/>
+      <c r="E63" s="15" t="n"/>
+      <c r="F63" s="15" t="n"/>
+      <c r="G63" s="15" t="n"/>
+      <c r="H63" s="16" t="n"/>
+      <c r="I63" s="15" t="n"/>
+      <c r="J63" s="15" t="n"/>
+      <c r="K63" s="15" t="n"/>
+      <c r="L63" s="15" t="n"/>
+      <c r="M63" s="16" t="n"/>
+      <c r="N63" s="15" t="n"/>
+      <c r="O63" s="15" t="n"/>
+      <c r="P63" s="15" t="n"/>
+      <c r="Q63" s="15" t="n"/>
+      <c r="R63" s="15" t="n"/>
+      <c r="S63" s="15" t="n"/>
+    </row>
+    <row r="64">
+      <c r="C64" s="15" t="n"/>
+      <c r="D64" s="15" t="n"/>
+      <c r="E64" s="15" t="n"/>
+      <c r="F64" s="15" t="n"/>
+      <c r="G64" s="15" t="n"/>
+      <c r="H64" s="16" t="n"/>
+      <c r="I64" s="15" t="n"/>
+      <c r="J64" s="15" t="n"/>
+      <c r="K64" s="15" t="n"/>
+      <c r="L64" s="15" t="n"/>
+      <c r="M64" s="16" t="n"/>
+      <c r="N64" s="15" t="n"/>
+      <c r="O64" s="15" t="n"/>
+      <c r="P64" s="15" t="n"/>
+      <c r="Q64" s="15" t="n"/>
+      <c r="R64" s="15" t="n"/>
+      <c r="S64" s="15" t="n"/>
+    </row>
+    <row r="65">
+      <c r="C65" s="15" t="n"/>
+      <c r="D65" s="15" t="n"/>
+      <c r="E65" s="15" t="n"/>
+      <c r="F65" s="15" t="n"/>
+      <c r="G65" s="15" t="n"/>
+      <c r="H65" s="16" t="n"/>
+      <c r="I65" s="15" t="n"/>
+      <c r="J65" s="15" t="n"/>
+      <c r="K65" s="15" t="n"/>
+      <c r="L65" s="15" t="n"/>
+      <c r="M65" s="16" t="n"/>
+      <c r="N65" s="15" t="n"/>
+      <c r="O65" s="15" t="n"/>
+      <c r="P65" s="15" t="n"/>
+      <c r="Q65" s="15" t="n"/>
+      <c r="R65" s="15" t="n"/>
+      <c r="S65" s="15" t="n"/>
+    </row>
+    <row r="66">
+      <c r="C66" s="15" t="n"/>
+      <c r="D66" s="15" t="n"/>
+      <c r="E66" s="15" t="n"/>
+      <c r="F66" s="15" t="n"/>
+      <c r="G66" s="15" t="n"/>
+      <c r="H66" s="16" t="n"/>
+      <c r="I66" s="15" t="n"/>
+      <c r="J66" s="15" t="n"/>
+      <c r="K66" s="15" t="n"/>
+      <c r="L66" s="15" t="n"/>
+      <c r="M66" s="16" t="n"/>
+      <c r="N66" s="15" t="n"/>
+      <c r="O66" s="15" t="n"/>
+      <c r="P66" s="15" t="n"/>
+      <c r="Q66" s="15" t="n"/>
+      <c r="R66" s="15" t="n"/>
+      <c r="S66" s="15" t="n"/>
+    </row>
+    <row r="67">
+      <c r="C67" s="15" t="n"/>
+      <c r="D67" s="15" t="n"/>
+      <c r="E67" s="15" t="n"/>
+      <c r="F67" s="15" t="n"/>
+      <c r="G67" s="15" t="n"/>
+      <c r="H67" s="16" t="n"/>
+      <c r="I67" s="15" t="n"/>
+      <c r="J67" s="15" t="n"/>
+      <c r="K67" s="15" t="n"/>
+      <c r="L67" s="15" t="n"/>
+      <c r="M67" s="16" t="n"/>
+      <c r="N67" s="15" t="n"/>
+      <c r="O67" s="15" t="n"/>
+      <c r="P67" s="15" t="n"/>
+      <c r="Q67" s="15" t="n"/>
+      <c r="R67" s="15" t="n"/>
+      <c r="S67" s="15" t="n"/>
+    </row>
+    <row r="68">
+      <c r="C68" s="15" t="n"/>
+      <c r="D68" s="15" t="n"/>
+      <c r="E68" s="15" t="n"/>
+      <c r="F68" s="15" t="n"/>
+      <c r="G68" s="15" t="n"/>
+      <c r="H68" s="16" t="n"/>
+      <c r="I68" s="15" t="n"/>
+      <c r="J68" s="15" t="n"/>
+      <c r="K68" s="15" t="n"/>
+      <c r="L68" s="15" t="n"/>
+      <c r="M68" s="16" t="n"/>
+      <c r="N68" s="15" t="n"/>
+      <c r="O68" s="15" t="n"/>
+      <c r="P68" s="15" t="n"/>
+      <c r="Q68" s="15" t="n"/>
+      <c r="R68" s="15" t="n"/>
+      <c r="S68" s="15" t="n"/>
+    </row>
+    <row r="69">
+      <c r="C69" s="15" t="n"/>
+      <c r="D69" s="15" t="n"/>
+      <c r="E69" s="15" t="n"/>
+      <c r="F69" s="15" t="n"/>
+      <c r="G69" s="15" t="n"/>
+      <c r="H69" s="16" t="n"/>
+      <c r="I69" s="15" t="n"/>
+      <c r="J69" s="15" t="n"/>
+      <c r="K69" s="15" t="n"/>
+      <c r="L69" s="15" t="n"/>
+      <c r="M69" s="16" t="n"/>
+      <c r="N69" s="15" t="n"/>
+      <c r="O69" s="15" t="n"/>
+      <c r="P69" s="15" t="n"/>
+      <c r="Q69" s="15" t="n"/>
+      <c r="R69" s="15" t="n"/>
+      <c r="S69" s="15" t="n"/>
+    </row>
+    <row r="70">
+      <c r="C70" s="15" t="n"/>
+      <c r="D70" s="15" t="n"/>
+      <c r="E70" s="15" t="n"/>
+      <c r="F70" s="15" t="n"/>
+      <c r="G70" s="15" t="n"/>
+      <c r="H70" s="16" t="n"/>
+      <c r="I70" s="15" t="n"/>
+      <c r="J70" s="15" t="n"/>
+      <c r="K70" s="15" t="n"/>
+      <c r="L70" s="15" t="n"/>
+      <c r="M70" s="16" t="n"/>
+      <c r="N70" s="15" t="n"/>
+      <c r="O70" s="15" t="n"/>
+      <c r="P70" s="15" t="n"/>
+      <c r="Q70" s="15" t="n"/>
+      <c r="R70" s="15" t="n"/>
+      <c r="S70" s="15" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="C10:S16"/>
+  <dataValidations count="4">
+    <dataValidation sqref="F11:F210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Approach,Environment,Schedule,Governance,Resourcing,Scope,Commercial,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K11:K210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pending,Approved,Rejected,Superseded"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q11:Q210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S11:S210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8060,7 +9708,7 @@
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Risks / Issues / Assumptions / Dependencies</t>
+          <t>Risks / Issues / Assumptions / Dependencies / Decisions</t>
         </is>
       </c>
       <c r="C6" s="17" t="inlineStr">
@@ -8089,7 +9737,7 @@
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t>Risks: Open / Mitigated / Closed. Issues: Open / Resolution in progress / Resolved / Closed. Dependencies: Open / Closed. Archived = Yes hides a row from the dashboard.</t>
+          <t>Risks: Open / Mitigated / Closed. Issues: Open / Resolution in progress / Resolved / Closed. Dependencies: Open / Closed. Decisions: Pending / Approved / Rejected / Superseded. Archived = Yes hides a row from the dashboard.</t>
         </is>
       </c>
     </row>

</xml_diff>